<commit_message>
feat: rediseno Glamour's Music estilo radio - hero full-screen + sticky bottom player
</commit_message>
<xml_diff>
--- a/Carga Masiva/22.05.2026.xlsx
+++ b/Carga Masiva/22.05.2026.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="38">
   <si>
     <t>Nombre</t>
   </si>
@@ -106,6 +106,33 @@
   </si>
   <si>
     <t>C:\AI\Antigravity\Tienda de Ropa\ropa\7060450010.jpeg</t>
+  </si>
+  <si>
+    <t>Camisa SANDRO</t>
+  </si>
+  <si>
+    <t>short SANDRO</t>
+  </si>
+  <si>
+    <t>Remera SANDRO</t>
+  </si>
+  <si>
+    <t>Remera</t>
+  </si>
+  <si>
+    <t>Camisa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">short </t>
+  </si>
+  <si>
+    <t>C:\AI\Antigravity\Tienda de Ropa\ropa\7060450011.jpg</t>
+  </si>
+  <si>
+    <t>C:\AI\Antigravity\Tienda de Ropa\ropa\7060450013.jpg</t>
+  </si>
+  <si>
+    <t>C:\AI\Antigravity\Tienda de Ropa\ropa\7060450012.jpg</t>
   </si>
 </sst>
 </file>
@@ -482,7 +509,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:S5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.5" bestFit="1" customWidth="1"/>
@@ -492,7 +519,7 @@
     <col min="5" max="5" width="5.875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="31.125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="47.75" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12.375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="14" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="6.375" bestFit="1" customWidth="1"/>
@@ -578,7 +605,7 @@
         <v>26</v>
       </c>
       <c r="E2">
-        <v>56000</v>
+        <v>58000</v>
       </c>
       <c r="F2">
         <v>58000</v>
@@ -620,13 +647,190 @@
         <v>1</v>
       </c>
       <c r="S2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3">
+        <v>59000</v>
+      </c>
+      <c r="F3">
+        <v>59000</v>
+      </c>
+      <c r="G3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H3" t="s">
+        <v>35</v>
+      </c>
+      <c r="I3" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3">
+        <v>1023450010</v>
+      </c>
+      <c r="K3" t="s">
+        <v>21</v>
+      </c>
+      <c r="L3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M3" t="s">
+        <v>23</v>
+      </c>
+      <c r="N3">
+        <v>1</v>
+      </c>
+      <c r="O3">
+        <v>1</v>
+      </c>
+      <c r="P3">
+        <v>1</v>
+      </c>
+      <c r="Q3">
+        <v>1</v>
+      </c>
+      <c r="R3">
+        <v>1</v>
+      </c>
+      <c r="S3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4">
+        <v>60000</v>
+      </c>
+      <c r="F4">
+        <v>60000</v>
+      </c>
+      <c r="G4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H4" t="s">
+        <v>37</v>
+      </c>
+      <c r="I4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J4">
+        <v>1023450010</v>
+      </c>
+      <c r="K4" t="s">
+        <v>21</v>
+      </c>
+      <c r="L4" t="s">
+        <v>22</v>
+      </c>
+      <c r="M4" t="s">
+        <v>23</v>
+      </c>
+      <c r="N4">
+        <v>1</v>
+      </c>
+      <c r="O4">
+        <v>1</v>
+      </c>
+      <c r="P4">
+        <v>1</v>
+      </c>
+      <c r="Q4">
+        <v>1</v>
+      </c>
+      <c r="R4">
+        <v>1</v>
+      </c>
+      <c r="S4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5">
+        <v>61000</v>
+      </c>
+      <c r="F5">
+        <v>61000</v>
+      </c>
+      <c r="G5" t="s">
+        <v>27</v>
+      </c>
+      <c r="H5" t="s">
+        <v>36</v>
+      </c>
+      <c r="I5" t="s">
+        <v>20</v>
+      </c>
+      <c r="J5">
+        <v>1023450010</v>
+      </c>
+      <c r="K5" t="s">
+        <v>21</v>
+      </c>
+      <c r="L5" t="s">
+        <v>22</v>
+      </c>
+      <c r="M5" t="s">
+        <v>23</v>
+      </c>
+      <c r="N5">
+        <v>1</v>
+      </c>
+      <c r="O5">
+        <v>1</v>
+      </c>
+      <c r="P5">
+        <v>1</v>
+      </c>
+      <c r="Q5">
+        <v>1</v>
+      </c>
+      <c r="R5">
+        <v>1</v>
+      </c>
+      <c r="S5">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:S1 C2 E2 I2 K2:L2" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:S1 C2 I2 K2:L2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>